<commit_message>
feat: add special holiday OT columns to payslip generation
</commit_message>
<xml_diff>
--- a/templates/payroll_template.xlsx
+++ b/templates/payroll_template.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL3"/>
+  <dimension ref="A1:AN3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,100 +521,110 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>SpecialHolidayOTHours</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>SpecialHolidayOTAmount</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>NightDiffHours</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>NightDiffAmount</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>OffsetHours</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>OffsetAmount</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>PaidLeaveHours</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>PaidLeaveAmount</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>AdjustmentEarnings</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>ThirteenthMonthPay</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>OthersEarnings</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>GrossIncome</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>SSSContribution</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>PhilhealthContribution</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>PagibigContribution</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>PagibigLoan</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>SSSLoan</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>WithholdingTax</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>AdjustmentDeductions</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>OthersDeductions</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>TotalDeductions</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>NetPay</t>
         </is>
@@ -698,51 +708,57 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
         <v>20</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Z2" t="n">
         <v>4500</v>
       </c>
-      <c r="Y2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0</v>
-      </c>
       <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="n">
         <v>1000</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AD2" t="n">
         <v>18000</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AE2" t="n">
         <v>500</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AF2" t="n">
         <v>300</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AG2" t="n">
         <v>200</v>
       </c>
-      <c r="AF2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG2" t="n">
-        <v>0</v>
-      </c>
       <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
         <v>300</v>
       </c>
-      <c r="AI2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ2" t="n">
+      <c r="AK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="n">
         <v>2000</v>
       </c>
-      <c r="AK2" t="n">
+      <c r="AM2" t="n">
         <v>1500</v>
       </c>
-      <c r="AL2" t="n">
+      <c r="AN2" t="n">
         <v>16500</v>
       </c>
     </row>
@@ -824,51 +840,57 @@
         <v>0</v>
       </c>
       <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
         <v>30</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Z3" t="n">
         <v>5500</v>
       </c>
-      <c r="Y3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>0</v>
-      </c>
       <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" t="n">
         <v>5000</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AD3" t="n">
         <v>21700</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AE3" t="n">
         <v>600</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AF3" t="n">
         <v>350</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AG3" t="n">
         <v>250</v>
       </c>
-      <c r="AF3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>0</v>
-      </c>
       <c r="AH3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ3" t="n">
         <v>400</v>
       </c>
-      <c r="AI3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ3" t="n">
+      <c r="AK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL3" t="n">
         <v>1000</v>
       </c>
-      <c r="AK3" t="n">
+      <c r="AM3" t="n">
         <v>1800</v>
       </c>
-      <c r="AL3" t="n">
+      <c r="AN3" t="n">
         <v>19900</v>
       </c>
     </row>

</xml_diff>